<commit_message>
update grade flutua preto
</commit_message>
<xml_diff>
--- a/DISPO.xlsx
+++ b/DISPO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NOT-MARCOS\Documents\GitHub\Catalogo-Olympikus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D3F40E-71B5-46D3-89F2-C884A8DFA384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D2EEF3B-D9EC-4DFB-8777-79412C30AAC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{D5233C47-2897-4F0E-9138-F4B2B2ED9B28}"/>
   </bookViews>
@@ -1717,13 +1717,27 @@
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="4"/>
-      <c r="S10" s="4"/>
-      <c r="T10" s="4"/>
-      <c r="U10" s="4"/>
-      <c r="V10" s="4"/>
-      <c r="W10" s="4"/>
+      <c r="Q10" s="4">
+        <v>1</v>
+      </c>
+      <c r="R10" s="4">
+        <v>2</v>
+      </c>
+      <c r="S10" s="4">
+        <v>2</v>
+      </c>
+      <c r="T10" s="4">
+        <v>3</v>
+      </c>
+      <c r="U10" s="4">
+        <v>2</v>
+      </c>
+      <c r="V10" s="4">
+        <v>1</v>
+      </c>
+      <c r="W10" s="4">
+        <v>1</v>
+      </c>
       <c r="X10" s="4"/>
       <c r="Y10" s="4"/>
       <c r="Z10" s="4"/>

</xml_diff>